<commit_message>
Updated Installers and instructions
Updated instructions on how to override Mac blocking, as well as updated the inputs and installers for those inputs.
</commit_message>
<xml_diff>
--- a/ChorelistGenerator_Output/ChoreList.xlsx
+++ b/ChorelistGenerator_Output/ChoreList.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="43">
   <si>
     <t>Chores To Do</t>
   </si>
@@ -26,115 +26,121 @@
     <t/>
   </si>
   <si>
+    <t>sweep or vacuum front of house &amp; mop</t>
+  </si>
+  <si>
+    <t>(entryway, dinning room, bedroom hall, hall leading to kitchen)</t>
+  </si>
+  <si>
+    <t>Hazel</t>
+  </si>
+  <si>
+    <t>clean microwave with spray cleaner &amp; clorox wipes</t>
+  </si>
+  <si>
+    <t>empty/add new litter in cat litter box in storage closet, shake out mat under storage closet cat litter box &amp; sweep and mop storage closet</t>
+  </si>
+  <si>
+    <t>dust fireplace &amp; mantel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sweep &amp; leaf blow front porch </t>
+  </si>
+  <si>
+    <t>clean boys bathroom pickup towels</t>
+  </si>
+  <si>
+    <t>take out trash, scrub shower, counter, and toilets. Remove hair from drain clog.</t>
+  </si>
+  <si>
+    <t>Jesse</t>
+  </si>
+  <si>
+    <t>clean &amp; wipe down stove &amp; counters by stove</t>
+  </si>
+  <si>
+    <t>wipe off bar</t>
+  </si>
+  <si>
+    <t>pick up living room</t>
+  </si>
+  <si>
+    <t>fold &amp; put away blankets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">empty cat litter box in dinning room and add new litter shake out mat and sweep in front of litter box </t>
+  </si>
+  <si>
+    <t>clean, dust &amp; straighten area on top of &amp; around Daisy's crate &amp; console bench under window</t>
+  </si>
+  <si>
+    <t>dust around and straighten living room desk area</t>
+  </si>
+  <si>
+    <t>take out trash</t>
+  </si>
+  <si>
+    <t>Ray</t>
+  </si>
+  <si>
+    <t>clean &amp; wipe down counters in pantry, and sweep or vacuum &amp; mop pantry</t>
+  </si>
+  <si>
+    <t>sweep &amp; leaf blow back porch on both sides of gate</t>
+  </si>
+  <si>
+    <t>clean, sweep &amp; mop kitchen bathroom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sweep or vacuum &amp; mop area by garage door </t>
+  </si>
+  <si>
+    <t>Sift cat litter box in Daddy &amp; Renee's Room &amp; add new litter if needed, shake out &amp; clean mat and vacuum in front of litter box</t>
+  </si>
+  <si>
+    <t>DO NOT EMPTY OUT OLD LITTER</t>
+  </si>
+  <si>
+    <t>sweep or vacuum living room &amp; mop</t>
+  </si>
+  <si>
+    <t>move Daisy's crate &amp; sofas</t>
+  </si>
+  <si>
+    <t>Ruby</t>
+  </si>
+  <si>
+    <t>sweep &amp; mop under bar stools &amp; area between sofa &amp; bar</t>
+  </si>
+  <si>
+    <t>wipe down counters &amp; island in kitchen</t>
+  </si>
+  <si>
+    <t>pick up area by garage door &amp; vacuum out drawer</t>
+  </si>
+  <si>
+    <t>sweep or vacuum &amp; mop kids bathroom</t>
+  </si>
+  <si>
+    <t>William</t>
+  </si>
+  <si>
     <t>sweep or vacuum &amp; mop kitchen</t>
   </si>
   <si>
     <t>including hall and area outside Daddy &amp; Renee's door, under counters &amp; in corners</t>
   </si>
   <si>
-    <t>Hazel</t>
-  </si>
-  <si>
-    <t>clean &amp; wipe down counters in pantry, and sweep or vacuum &amp; mop pantry</t>
+    <t>dust in the entry way and dinning room including desk area, empty trash can next to desk</t>
+  </si>
+  <si>
+    <t>wipe off dining table</t>
+  </si>
+  <si>
+    <t>clean kitchen garbage cans area</t>
   </si>
   <si>
     <t>dust windows and doors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sweep or vacuum &amp; mop area by garage door </t>
-  </si>
-  <si>
-    <t xml:space="preserve">sweep &amp; leaf blow front porch </t>
-  </si>
-  <si>
-    <t>clean boys bathroom pickup towels</t>
-  </si>
-  <si>
-    <t>take out trash, scrub shower and counter.</t>
-  </si>
-  <si>
-    <t>Jesse</t>
-  </si>
-  <si>
-    <t>clean, sweep &amp; mop kitchen bathroom</t>
-  </si>
-  <si>
-    <t>take out trash</t>
-  </si>
-  <si>
-    <t>sweep &amp; mop under bar stools &amp; area between sofa &amp; bar</t>
-  </si>
-  <si>
-    <t>pick up area by garage door &amp; vacuum out drawer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">empty cat litter box in dinning room and add new litter shake out mat and sweep in front of litter box </t>
-  </si>
-  <si>
-    <t>dust around and straighten living room desk area</t>
-  </si>
-  <si>
-    <t>Ray</t>
-  </si>
-  <si>
-    <t>clean &amp; wipe down stove &amp; counters by stove</t>
-  </si>
-  <si>
-    <t>wipe down counters &amp; island in kitchen</t>
-  </si>
-  <si>
-    <t>clean microwave with spray cleaner &amp; clorox wipes</t>
-  </si>
-  <si>
-    <t>empty/add new litter in cat litter box in storage closet, shake out mat under storage closet cat litter box &amp; sweep and mop storage closet</t>
-  </si>
-  <si>
-    <t>clean, dust &amp; straighten area on top of &amp; around Daisy's crate &amp; console bench under window</t>
-  </si>
-  <si>
-    <t>sweep or vacuum front of house &amp; mop</t>
-  </si>
-  <si>
-    <t>(entryway, dinning room, bedroom hall, hall leading to kitchen)</t>
-  </si>
-  <si>
-    <t>Ruby</t>
-  </si>
-  <si>
-    <t>pick up living room</t>
-  </si>
-  <si>
-    <t>fold &amp; put away blankets</t>
-  </si>
-  <si>
-    <t>clean kitchen garbage cans area</t>
-  </si>
-  <si>
-    <t>sweep or vacuum &amp; mop kids bathroom</t>
-  </si>
-  <si>
-    <t>William</t>
-  </si>
-  <si>
-    <t>sweep &amp; leaf blow back porch on both sides of gate</t>
-  </si>
-  <si>
-    <t>dust in the entry way and dinning room including desk area, empty trash can next to desk</t>
-  </si>
-  <si>
-    <t>wipe off dining table</t>
-  </si>
-  <si>
-    <t>wipe off bar</t>
-  </si>
-  <si>
-    <t>dust fireplace &amp; mantel</t>
-  </si>
-  <si>
-    <t>Sift cat litter box in Daddy &amp; Renee's Room &amp; add new litter if needed, shake out &amp; clean mat and vacuum in front of litter box</t>
-  </si>
-  <si>
-    <t>DO NOT EMPTY OUT OLD LITTER</t>
   </si>
 </sst>
 </file>
@@ -235,7 +241,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="43.0" customWidth="true"/>
@@ -358,7 +364,7 @@
         <v>14</v>
       </c>
       <c r="B9" t="s" s="6">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="C9" t="s" s="3">
         <v>13</v>
@@ -369,7 +375,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="3">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s" s="6">
         <v>3</v>
@@ -383,10 +389,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="3">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s" s="6">
         <v>17</v>
-      </c>
-      <c r="B11" t="s" s="6">
-        <v>3</v>
       </c>
       <c r="C11" t="s" s="3">
         <v>13</v>
@@ -396,56 +402,56 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="s" s="4">
+      <c r="A12" t="s" s="3">
         <v>18</v>
       </c>
-      <c r="B12" t="s" s="7">
-        <v>3</v>
-      </c>
-      <c r="C12" t="s" s="4">
+      <c r="B12" t="s" s="6">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s" s="3">
         <v>13</v>
       </c>
-      <c r="D12" t="s" s="4">
+      <c r="D12" t="s" s="3">
         <v>3</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="s" s="2">
+      <c r="A13" t="s" s="4">
         <v>19</v>
       </c>
-      <c r="B13" t="s" s="5">
-        <v>15</v>
-      </c>
-      <c r="C13" t="s" s="2">
+      <c r="B13" t="s" s="7">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s" s="4">
+        <v>13</v>
+      </c>
+      <c r="D13" t="s" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="2">
         <v>20</v>
       </c>
-      <c r="D13" t="s" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="3">
+      <c r="B14" t="s" s="5">
         <v>21</v>
       </c>
-      <c r="B14" t="s" s="6">
-        <v>3</v>
-      </c>
-      <c r="C14" t="s" s="3">
-        <v>20</v>
-      </c>
-      <c r="D14" t="s" s="3">
+      <c r="C14" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D14" t="s" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="3">
+        <v>23</v>
+      </c>
+      <c r="B15" t="s" s="6">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s" s="3">
         <v>22</v>
-      </c>
-      <c r="B15" t="s" s="6">
-        <v>3</v>
-      </c>
-      <c r="C15" t="s" s="3">
-        <v>20</v>
       </c>
       <c r="D15" t="s" s="3">
         <v>3</v>
@@ -453,13 +459,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="3">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16" t="s" s="6">
         <v>3</v>
       </c>
       <c r="C16" t="s" s="3">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D16" t="s" s="3">
         <v>3</v>
@@ -467,113 +473,113 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="3">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s" s="6">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="C17" t="s" s="3">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D17" t="s" s="3">
         <v>3</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="s" s="4">
-        <v>25</v>
-      </c>
-      <c r="B18" t="s" s="7">
-        <v>3</v>
-      </c>
-      <c r="C18" t="s" s="4">
-        <v>20</v>
-      </c>
-      <c r="D18" t="s" s="4">
+      <c r="A18" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="B18" t="s" s="6">
+        <v>3</v>
+      </c>
+      <c r="C18" t="s" s="3">
+        <v>22</v>
+      </c>
+      <c r="D18" t="s" s="3">
         <v>3</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="s" s="2">
-        <v>26</v>
-      </c>
-      <c r="B19" t="s" s="5">
+      <c r="A19" t="s" s="4">
         <v>27</v>
       </c>
-      <c r="C19" t="s" s="2">
+      <c r="B19" t="s" s="7">
         <v>28</v>
       </c>
-      <c r="D19" t="s" s="2">
+      <c r="C19" t="s" s="4">
+        <v>22</v>
+      </c>
+      <c r="D19" t="s" s="4">
         <v>3</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="s" s="3">
+      <c r="A20" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="B20" t="s" s="6">
+      <c r="B20" t="s" s="5">
         <v>30</v>
       </c>
-      <c r="C20" t="s" s="3">
-        <v>28</v>
-      </c>
-      <c r="D20" t="s" s="3">
+      <c r="C20" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="D20" t="s" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="s" s="4">
+      <c r="A21" t="s" s="3">
+        <v>32</v>
+      </c>
+      <c r="B21" t="s" s="6">
+        <v>3</v>
+      </c>
+      <c r="C21" t="s" s="3">
         <v>31</v>
       </c>
-      <c r="B21" t="s" s="7">
-        <v>3</v>
-      </c>
-      <c r="C21" t="s" s="4">
-        <v>28</v>
-      </c>
-      <c r="D21" t="s" s="4">
+      <c r="D21" t="s" s="3">
         <v>3</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="B22" t="s" s="5">
-        <v>3</v>
-      </c>
-      <c r="C22" t="s" s="2">
+      <c r="A22" t="s" s="3">
         <v>33</v>
       </c>
-      <c r="D22" t="s" s="2">
+      <c r="B22" t="s" s="6">
+        <v>3</v>
+      </c>
+      <c r="C22" t="s" s="3">
+        <v>31</v>
+      </c>
+      <c r="D22" t="s" s="3">
         <v>3</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="s" s="3">
+      <c r="A23" t="s" s="4">
         <v>34</v>
       </c>
-      <c r="B23" t="s" s="6">
-        <v>3</v>
-      </c>
-      <c r="C23" t="s" s="3">
-        <v>33</v>
-      </c>
-      <c r="D23" t="s" s="3">
+      <c r="B23" t="s" s="7">
+        <v>3</v>
+      </c>
+      <c r="C23" t="s" s="4">
+        <v>31</v>
+      </c>
+      <c r="D23" t="s" s="4">
         <v>3</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="s" s="3">
+      <c r="A24" t="s" s="2">
         <v>35</v>
       </c>
-      <c r="B24" t="s" s="6">
+      <c r="B24" t="s" s="5">
+        <v>3</v>
+      </c>
+      <c r="C24" t="s" s="2">
         <v>36</v>
       </c>
-      <c r="C24" t="s" s="3">
-        <v>33</v>
-      </c>
-      <c r="D24" t="s" s="3">
+      <c r="D24" t="s" s="2">
         <v>3</v>
       </c>
     </row>
@@ -582,10 +588,10 @@
         <v>37</v>
       </c>
       <c r="B25" t="s" s="6">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="C25" t="s" s="3">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D25" t="s" s="3">
         <v>3</v>
@@ -593,29 +599,43 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="3">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B26" t="s" s="6">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="C26" t="s" s="3">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D26" t="s" s="3">
         <v>3</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="s" s="4">
-        <v>39</v>
-      </c>
-      <c r="B27" t="s" s="7">
-        <v>40</v>
-      </c>
-      <c r="C27" t="s" s="4">
-        <v>33</v>
-      </c>
-      <c r="D27" t="s" s="4">
+      <c r="A27" t="s" s="3">
+        <v>41</v>
+      </c>
+      <c r="B27" t="s" s="6">
+        <v>3</v>
+      </c>
+      <c r="C27" t="s" s="3">
+        <v>36</v>
+      </c>
+      <c r="D27" t="s" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="4">
+        <v>42</v>
+      </c>
+      <c r="B28" t="s" s="7">
+        <v>3</v>
+      </c>
+      <c r="C28" t="s" s="4">
+        <v>36</v>
+      </c>
+      <c r="D28" t="s" s="4">
         <v>3</v>
       </c>
     </row>

</xml_diff>